<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@8e5f0fbafc5dad8ef368bfff0f513b91200abae6 🚀
</commit_message>
<xml_diff>
--- a/ValueSet-DocumentLOINCCodelist.xlsx
+++ b/ValueSet-DocumentLOINCCodelist.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="42">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-10-03T16:43:05+00:00</t>
+    <t>2024-10-03T16:45:10+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -85,6 +85,9 @@
   </si>
   <si>
     <t>Description</t>
+  </si>
+  <si>
+    <t>Docuemnt Class en Type LOINC codes die we vinden zonder display, zodat we wel een display in Nederlands kunnen tonen</t>
   </si>
   <si>
     <t>Purpose</t>
@@ -376,28 +379,30 @@
       <c r="A13" t="s" s="2">
         <v>23</v>
       </c>
-      <c r="B13" s="2"/>
+      <c r="B13" t="s" s="2">
+        <v>24</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B14" s="2"/>
     </row>
     <row r="15">
       <c r="A15" t="s" s="2">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="2">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -416,7 +421,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="1">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s" s="1">
         <v>23</v>
@@ -424,50 +429,50 @@
     </row>
     <row r="2">
       <c r="A2" t="s" s="2">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B2" t="s" s="2">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="2">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B5" t="s" s="2">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="2">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B6" t="s" s="2">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="2">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B7" t="s" s="2">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@7d41f181590f6b1bfc7eeda5c0dea21ee6dae029 🚀
</commit_message>
<xml_diff>
--- a/ValueSet-DocumentLOINCCodelist.xlsx
+++ b/ValueSet-DocumentLOINCCodelist.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-01-02T12:37:15+00:00</t>
+    <t>2025-01-05T10:27:23+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -96,7 +96,7 @@
     <t>Copyright</t>
   </si>
   <si>
-    <t>This value set includes content from LOINC</t>
+    <t>This material contains content from LOINC (http://loinc.org). LOINC is copyright © 1995-2020, Regenstrief Institute, Inc. and the Logical Observation Identifiers Names and Codes (LOINC) Committee and is available at no cost under the license at http://loinc.org/license. LOINC® is a registered United States trademark of Regenstrief Institute, Inc</t>
   </si>
   <si>
     <t>Immutable</t>

</xml_diff>